<commit_message>
Add MTK supplementary unit to shipment 581338 summary
KN 5903 20 10 takes m² (MTK) as its supplementary unit. MTK = 836,
from the client's e-mail of 17 Aug 2026 and consistent with
550 running metres x 1.52 m width.

Adds a "Doplňková jednotka (MTK)" and "Množství MTK (m²)" column to
the summary sheet plus an explanatory row on the notes sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017iVJrUAWNWemUfPXCGjwoo
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Singing_Rock_581338.xlsx
+++ b/output/HS_Code_Summary_Singing_Rock_581338.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -505,12 +505,14 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -690,35 +692,45 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
+          <t>Doplňková jednotka (MTK)</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Množství MTK (m²)</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
           <t>Cena / celní hodnota</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>Měna</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>INCOTERM (termín + místo)</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="O15" s="3" t="inlineStr">
         <is>
           <t>Preferenční původ (COO)</t>
         </is>
       </c>
-      <c r="N15" s="3" t="inlineStr">
+      <c r="P15" s="3" t="inlineStr">
         <is>
           <t>Poznámka</t>
         </is>
@@ -756,35 +768,43 @@
           <t>550 M (836 m², 6 rolí)</t>
         </is>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>MTK</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>836</v>
+      </c>
+      <c r="J16" s="6" t="n">
         <v>3025</v>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>FOB Busan</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>Není předmětem CBAM (kap. 59 – textil není v příloze I nařízení CBAM). Příjemce je v registru: Y128, povolení CBAM-CZ-2026-LIR35383169093, EORI CZ26000954, datum vydání 2026-06-08.</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Nezjištěno žádné antidumpingové opatření pro KN 5903 20 s původem v Korejské republice.</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>ANO – preferenční věta na faktuře i na packing listu (korejské celní oprávnění č. 010-11-230876). REX číslo NENÍ na faktuře uvedeno.</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>HS kód převzat z popisu zboží od klienta (59032010). B/L uvádí 5903.20-0000 a popis „PU COATED FABRIC“ – viz list Poznámky a nesrovnalosti.</t>
         </is>
@@ -807,10 +827,18 @@
           <t>550 M</t>
         </is>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>MTK</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>836</v>
+      </c>
+      <c r="J17" s="8" t="n">
         <v>3025</v>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -818,18 +846,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="C12:N12"/>
-    <mergeCell ref="C6:N6"/>
-    <mergeCell ref="C10:N10"/>
-    <mergeCell ref="C11:N11"/>
-    <mergeCell ref="C5:N5"/>
-    <mergeCell ref="C7:N7"/>
-    <mergeCell ref="C8:N8"/>
-    <mergeCell ref="C9:N9"/>
-    <mergeCell ref="C13:N13"/>
-    <mergeCell ref="C3:N3"/>
-    <mergeCell ref="C4:N4"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="C9:P9"/>
+    <mergeCell ref="C3:P3"/>
+    <mergeCell ref="C8:P8"/>
+    <mergeCell ref="C4:P4"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="C12:P12"/>
+    <mergeCell ref="C6:P6"/>
+    <mergeCell ref="C7:P7"/>
+    <mergeCell ref="C10:P10"/>
+    <mergeCell ref="C11:P11"/>
+    <mergeCell ref="C5:P5"/>
+    <mergeCell ref="C13:P13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -841,7 +869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1043,18 +1071,35 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
+    <row r="14" ht="65" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
+          <t>DOPLŇKOVÁ JEDNOTKA (MTK)</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>836 m²</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Pro KN 5903 20 10 je doplňkovou jednotkou metr čtvereční — kód MTK. Pro tuto zásilku činí MTK = 836 m². Údaj uvádí klientka přímo v e-mailu ze 17. 8. 2026 („Jedná se o 836m2.“) a souhlasí s přepočtem 550 bm × šíře 1,52 m = 836 m² (šíře odpovídá rozměru rolí 152 × 152 × 15 cm z původní poptávky). Do JSD se tedy vedle čisté hmotnosti 219 kg uvádí doplňková jednotka 836 MTK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
           <t>MNOŽSTVÍ A HMOTNOSTI</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>ÚPLNÉ</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Packing list: 550 M, 6 rolí, net 219 kg, gross 221 kg. Klient v e-mailu uvádí 836 m², což odpovídá 550 m × šíře 1,52 m (rozměr rolí 152 × 152 × 15 cm). Všechny povinné sloupce (HS kód, popis, čistá hmotnost, hrubá hmotnost, množství, cena) jsou v podkladech k dispozici — nic nechybí.</t>
         </is>

</xml_diff>